<commit_message>
Import: read first sheet of workbook instead of requiring 'fig1' name
</commit_message>
<xml_diff>
--- a/test_inbound1.xlsx
+++ b/test_inbound1.xlsx
@@ -8,16 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\warehouse_mgr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC490E78-75C1-4749-9A23-CFEE4F0CB24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0196397-9626-45CD-ACB3-70D0FCBBF618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7051007A-6A33-46F4-ACD3-D45E201BBF65}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A48A8ABB-CF4D-4D2F-97BA-E472414F5723}"/>
   </bookViews>
   <sheets>
-    <sheet name="fig1" sheetId="1" r:id="rId1"/>
-    <sheet name="fig2" sheetId="2" r:id="rId2"/>
-    <sheet name="fig3" sheetId="3" r:id="rId3"/>
-    <sheet name="fig4" sheetId="4" r:id="rId4"/>
-    <sheet name="fig5" sheetId="5" r:id="rId5"/>
+    <sheet name="工作表1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
   <si>
     <t>到貨日期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -83,10 +79,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>備註</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>陳令佳</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -107,6 +99,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>COMPACTLOGIX EXPANSION CABLE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>1769-OF4CI</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -115,23 +111,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>Compactlogix 32 Point Digital Input</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>1769-OB32</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>32 POINT 24 VDC OUTPUT MODULE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>1769-IF18</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>COMPACTLOGIX EXPANSION CABLE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Compactlogix 32 Point Digital Input</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>32 POINT 24 VDC OUTPUT MODULE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -200,325 +192,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>161375</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="圖片 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72B245AC-55B2-45B1-97E5-8CDA815325EF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="2352675"/>
-          <a:ext cx="14401800" cy="6190700"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>569759</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>47073</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="圖片 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E5E72FF1-9717-4C28-896F-87AD3D112F06}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="5057775"/>
-          <a:ext cx="13923809" cy="4419048"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>479478</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="圖片 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD70046A-BD83-423A-A12E-2EB7492EF19B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="14195478" cy="1809750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>3922</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="圖片 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB7221F9-267B-46D4-BBF7-F910DA0C2BE2}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="15091522" cy="1895475"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>9524</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>74326</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="圖片 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3825C949-E5AF-4113-8D20-811ADF57CE5A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="14411324" cy="6151276"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>6556</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="圖片 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F14D6C2-65B8-44C0-862F-55032910E2F4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="16465756" cy="2657475"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -817,15 +490,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9386561-AA4A-4BA8-94C9-2C2036F3E414}">
-  <dimension ref="A1:K7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DEB820-F7AC-4A8C-99B5-D02FB059DDD1}">
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.75" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -856,22 +525,19 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46133</v>
       </c>
       <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
       </c>
       <c r="G2">
         <v>11</v>
@@ -880,24 +546,24 @@
         <v>20260320004</v>
       </c>
       <c r="J2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46133</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
       <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
         <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
       </c>
       <c r="G3">
         <v>104</v>
@@ -906,18 +572,18 @@
         <v>20260320004</v>
       </c>
       <c r="J3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>46133</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
@@ -929,24 +595,24 @@
         <v>20260320004</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>46133</v>
       </c>
       <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
         <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
       </c>
       <c r="D5" t="s">
         <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G5">
         <v>780</v>
@@ -955,24 +621,24 @@
         <v>20260320004</v>
       </c>
       <c r="J5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46133</v>
       </c>
       <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G6">
         <v>659</v>
@@ -981,21 +647,21 @@
         <v>20260320004</v>
       </c>
       <c r="J6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>46133</v>
       </c>
       <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G7">
         <v>42</v>
@@ -1004,57 +670,11 @@
         <v>20260320004</v>
       </c>
       <c r="J7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12275845-D158-4BFA-A48E-D8444657E48D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C98F33-18CC-4494-A620-F9C04D0A93FB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4DDE54-1876-4544-9F36-6E8AEF3B611C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AF64FBC-6125-4242-B571-73683A669021}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Import: capture 出貨對象/供應商 column + add import button to inbound page
- FIG1_HEADERS now includes 出貨對象 (accepts 供應商 as alias)
- Importer groups by (date, PO, signer, supplier) and writes supplier_id
- Result table and dry-run preview show supplier column
- Inbound list page gets a '📥 從 Excel 匯入' button
</commit_message>
<xml_diff>
--- a/test_inbound1.xlsx
+++ b/test_inbound1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\warehouse_mgr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0196397-9626-45CD-ACB3-70D0FCBBF618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8E14507-D1E1-454B-A121-BD5C2AFED548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A48A8ABB-CF4D-4D2F-97BA-E472414F5723}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="30">
   <si>
     <t>到貨日期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -124,6 +124,38 @@
   </si>
   <si>
     <t>1769-IF18</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>供應商</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>所羅門股份有限公司</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>普得企業股份有限公司</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Schneider</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MGPM-8330</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>集合式電錶 PM5330</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>蔡培君</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1E右側</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -491,10 +523,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DEB820-F7AC-4A8C-99B5-D02FB059DDD1}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.75" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -502,31 +538,34 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46133</v>
       </c>
@@ -534,22 +573,25 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>11</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>20260320004</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46133</v>
       </c>
@@ -557,25 +599,28 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>104</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>20260320004</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>46133</v>
       </c>
@@ -583,22 +628,25 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>184</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>20260320004</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>46133</v>
       </c>
@@ -606,25 +654,28 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>18</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>780</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>20260320004</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46133</v>
       </c>
@@ -632,25 +683,28 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>19</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>20</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>659</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>20260320004</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>46133</v>
       </c>
@@ -658,19 +712,54 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>21</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>42</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>20260320004</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>46135</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8">
+        <v>50</v>
+      </c>
+      <c r="I8" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8">
+        <v>20260326003</v>
+      </c>
+      <c r="K8" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove '取消回傳總部' button and photo_unsend endpoint
</commit_message>
<xml_diff>
--- a/test_inbound1.xlsx
+++ b/test_inbound1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\warehouse_mgr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8E14507-D1E1-454B-A121-BD5C2AFED548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{59CFA669-CBFF-4C96-9E38-E92881264745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A48A8ABB-CF4D-4D2F-97BA-E472414F5723}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="36">
   <si>
     <t>到貨日期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -55,10 +55,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>產品敘述</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>序號</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -99,10 +95,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>COMPACTLOGIX EXPANSION CABLE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>1769-OF4CI</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -111,18 +103,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Compactlogix 32 Point Digital Input</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>1769-OB32</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>32 POINT 24 VDC OUTPUT MODULE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>1769-IF18</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -147,16 +131,49 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>集合式電錶 PM5330</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>蔡培君</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>1E右側</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SN:CD088A0T26210004</t>
+  </si>
+  <si>
+    <t>勁傑_蕭碧</t>
+  </si>
+  <si>
+    <t>22C-D088A103</t>
+  </si>
+  <si>
+    <t>倉庫中間地板</t>
+  </si>
+  <si>
+    <t>22C-D142A103</t>
+  </si>
+  <si>
+    <t>SN:CD142A0T26210010</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SN:CD142A0T26210011</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SN:CD142A0T26210012</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SN:CD142A0T26210013</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>22C-D208A103</t>
+  </si>
+  <si>
+    <t>SN:CD208A0T26200006</t>
   </si>
 </sst>
 </file>
@@ -523,14 +540,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DEB820-F7AC-4A8C-99B5-D02FB059DDD1}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -538,7 +555,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -561,209 +578,351 @@
       <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46133</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2">
+        <v>11</v>
+      </c>
+      <c r="I2">
+        <v>20260320004</v>
+      </c>
+      <c r="J2" t="s">
         <v>12</v>
       </c>
-      <c r="H2">
-        <v>11</v>
-      </c>
-      <c r="J2">
-        <v>20260320004</v>
-      </c>
-      <c r="K2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46133</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3">
+        <v>13</v>
+      </c>
+      <c r="G3">
         <v>104</v>
       </c>
-      <c r="J3">
+      <c r="I3">
         <v>20260320004</v>
       </c>
-      <c r="K3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>46133</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4">
+        <v>14</v>
+      </c>
+      <c r="G4">
         <v>184</v>
       </c>
-      <c r="J4">
+      <c r="I4">
         <v>20260320004</v>
       </c>
-      <c r="K4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>46133</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5">
+        <v>15</v>
+      </c>
+      <c r="G5">
         <v>780</v>
       </c>
-      <c r="J5">
+      <c r="I5">
         <v>20260320004</v>
       </c>
-      <c r="K5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46133</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6">
+        <v>16</v>
+      </c>
+      <c r="G6">
         <v>659</v>
       </c>
-      <c r="J6">
+      <c r="I6">
         <v>20260320004</v>
       </c>
-      <c r="K6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>46133</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7">
+        <v>17</v>
+      </c>
+      <c r="G7">
         <v>42</v>
       </c>
-      <c r="J7">
+      <c r="I7">
         <v>20260320004</v>
       </c>
-      <c r="K7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>46135</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8">
+        <v>20260326003</v>
+      </c>
+      <c r="J8" t="s">
         <v>24</v>
       </c>
-      <c r="D8" t="s">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" t="s">
         <v>25</v>
       </c>
-      <c r="E8" t="s">
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
         <v>26</v>
       </c>
-      <c r="F8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8">
-        <v>50</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="J10" t="s">
         <v>28</v>
       </c>
-      <c r="J8">
-        <v>20260326003</v>
-      </c>
-      <c r="K8" t="s">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
         <v>29</v>
+      </c>
+      <c r="F11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="J11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="J12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="J13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="J14" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>